<commit_message>
initial fix for menus
</commit_message>
<xml_diff>
--- a/basic_page.xlsx
+++ b/basic_page.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="17">
   <si>
     <t>CPT</t>
   </si>
@@ -44,25 +44,16 @@
     <t>menu not found on wordpress</t>
   </si>
   <si>
-    <t>/aac/</t>
-  </si>
-  <si>
-    <t>Menu matched</t>
-  </si>
-  <si>
-    <t>/accounting/</t>
-  </si>
-  <si>
-    <t>Menu not found on drupal and wp content is similar</t>
-  </si>
-  <si>
     <t>/rotc/</t>
   </si>
   <si>
     <t>Menu items missing on wordpress</t>
   </si>
   <si>
-    <t>/academic-program-finder/biochemistry/</t>
+    <t>biochemistry</t>
+  </si>
+  <si>
+    <t>/biochemistry</t>
   </si>
   <si>
     <t>"HOME" menu item missing from menu</t>
@@ -87,6 +78,9 @@
   </si>
   <si>
     <t>/geology/prospective_students/</t>
+  </si>
+  <si>
+    <t>/education/admissions</t>
   </si>
 </sst>
 </file>
@@ -1066,7 +1060,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultColWidth="8.8359375" defaultRowHeight="16.8" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
@@ -1093,7 +1087,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" ht="34" spans="1:3">
+    <row r="3" ht="20.8" spans="1:3">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -1104,81 +1098,67 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" ht="101" spans="1:3">
+    <row r="4" ht="20.8" spans="1:3">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="2" t="s">
         <v>7</v>
       </c>
+      <c r="C4" s="3" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="5" ht="101" spans="1:3">
+    <row r="5" ht="34" spans="1:3">
       <c r="A5" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
-    <row r="6" ht="20.8" spans="1:3">
-      <c r="A6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="3" t="s">
+    <row r="6" ht="21" customHeight="1" spans="1:3">
+      <c r="A6" t="s">
         <v>11</v>
       </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="7" ht="34" spans="1:3">
-      <c r="A7" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="2" t="s">
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
         <v>13</v>
       </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" t="s">
+        <v>14</v>
+      </c>
     </row>
-    <row r="8" ht="21" customHeight="1" spans="1:3">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" t="s">
         <v>14</v>
       </c>
-      <c r="B8" t="s">
-        <v>14</v>
-      </c>
-      <c r="C8" t="s">
-        <v>15</v>
-      </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:2">
       <c r="A9" t="s">
         <v>16</v>
       </c>
       <c r="B9" t="s">
         <v>16</v>
-      </c>
-      <c r="C9" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" t="s">
-        <v>18</v>
-      </c>
-      <c r="C10" t="s">
-        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>